<commit_message>
adding style and image logo to page
</commit_message>
<xml_diff>
--- a/App_Data/AcademicCalendar.xlsx
+++ b/App_Data/AcademicCalendar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elie.tawk\source\repos\AcademicCalendarProject\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{77749D28-A6C8-4170-87E0-B9B1343FA513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5FDB651-EE90-4FA8-9446-607894A9B02E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{53C95AB7-0C09-47B5-9AE8-636C0202DA36}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="36">
   <si>
     <t>EventTitle</t>
   </si>
@@ -55,6 +55,96 @@
   </si>
   <si>
     <t>IsActive</t>
+  </si>
+  <si>
+    <t>USEK Entrance Exam for regular admission</t>
+  </si>
+  <si>
+    <t>Entrance exam for regular admission applicants</t>
+  </si>
+  <si>
+    <t>Exams</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Deadline for Course Withdrawal (W)</t>
+  </si>
+  <si>
+    <t>Last day to withdraw from course</t>
+  </si>
+  <si>
+    <t>Deadlines</t>
+  </si>
+  <si>
+    <t>Second Comprehensive Exam for postgraduate applicants</t>
+  </si>
+  <si>
+    <t>Comprehensive exam for postgraduate applicants</t>
+  </si>
+  <si>
+    <t>Deadline to settle 2nd and final installment</t>
+  </si>
+  <si>
+    <t>Final payment deadline for summer session</t>
+  </si>
+  <si>
+    <t>Application of the financial penalty</t>
+  </si>
+  <si>
+    <t>Financial penalty starts after deadline</t>
+  </si>
+  <si>
+    <t>Readmission request deadline</t>
+  </si>
+  <si>
+    <t>Deadline to submit readmission request</t>
+  </si>
+  <si>
+    <t>Entrance Exam for Engineering programs</t>
+  </si>
+  <si>
+    <t>Entrance exam for engineering applicants</t>
+  </si>
+  <si>
+    <t>Online Application Deactivation</t>
+  </si>
+  <si>
+    <t>Online application closes for Fall semester</t>
+  </si>
+  <si>
+    <t>Academic</t>
+  </si>
+  <si>
+    <t>Final Exams Begin</t>
+  </si>
+  <si>
+    <t>Summer session final exams begin</t>
+  </si>
+  <si>
+    <t>Summer Session Ends</t>
+  </si>
+  <si>
+    <t>End of summer academic session</t>
+  </si>
+  <si>
+    <t>Registration Opens</t>
+  </si>
+  <si>
+    <t>Registration starts for Fall semester</t>
+  </si>
+  <si>
+    <t>Registration</t>
+  </si>
+  <si>
+    <t>Assumption Day</t>
+  </si>
+  <si>
+    <t>Official holiday</t>
+  </si>
+  <si>
+    <t>Holidays</t>
   </si>
 </sst>
 </file>
@@ -98,12 +188,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -418,14 +514,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40EBC4DB-878C-491D-A5FD-57243F5A39BE}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="2"/>
-    <col min="4" max="4" width="8.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="48.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5546875" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="8.88671875" style="2"/>
   </cols>
@@ -450,6 +545,224 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="4">
+        <v>46205</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="4">
+        <v>46209</v>
+      </c>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="4">
+        <v>46211</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="4">
+        <v>46212</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="4">
+        <v>46213</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="4">
+        <v>46216</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="4">
+        <v>46217</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="4">
+        <v>46218</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="4">
+        <v>46223</v>
+      </c>
+      <c r="D10" s="4">
+        <v>46228</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="4">
+        <v>46234</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="4">
+        <v>46239</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="4">
+        <v>46249</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Adjusted list view each month a card and adjusted excel table
</commit_message>
<xml_diff>
--- a/App_Data/AcademicCalendar.xlsx
+++ b/App_Data/AcademicCalendar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elie.tawk\source\repos\AcademicCalendarProject\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5FDB651-EE90-4FA8-9446-607894A9B02E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{879C70B6-D5B2-4C5F-A3EB-80D4745EA5CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{53C95AB7-0C09-47B5-9AE8-636C0202DA36}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="46">
   <si>
     <t>EventTitle</t>
   </si>
@@ -45,21 +45,12 @@
     <t>EventDescription</t>
   </si>
   <si>
-    <t>StartDate</t>
-  </si>
-  <si>
-    <t>EndDate</t>
-  </si>
-  <si>
     <t>Category</t>
   </si>
   <si>
     <t>IsActive</t>
   </si>
   <si>
-    <t>USEK Entrance Exam for regular admission</t>
-  </si>
-  <si>
     <t>Entrance exam for regular admission applicants</t>
   </si>
   <si>
@@ -78,24 +69,6 @@
     <t>Deadlines</t>
   </si>
   <si>
-    <t>Second Comprehensive Exam for postgraduate applicants</t>
-  </si>
-  <si>
-    <t>Comprehensive exam for postgraduate applicants</t>
-  </si>
-  <si>
-    <t>Deadline to settle 2nd and final installment</t>
-  </si>
-  <si>
-    <t>Final payment deadline for summer session</t>
-  </si>
-  <si>
-    <t>Application of the financial penalty</t>
-  </si>
-  <si>
-    <t>Financial penalty starts after deadline</t>
-  </si>
-  <si>
     <t>Readmission request deadline</t>
   </si>
   <si>
@@ -145,6 +118,63 @@
   </si>
   <si>
     <t>Holidays</t>
+  </si>
+  <si>
+    <t>ULS Entrance Exam for regular admission</t>
+  </si>
+  <si>
+    <t>Fall Registration Opens</t>
+  </si>
+  <si>
+    <t>Registration for Fall semester</t>
+  </si>
+  <si>
+    <t>Fall Semester Begins</t>
+  </si>
+  <si>
+    <t>Classes begin</t>
+  </si>
+  <si>
+    <t>Add Drop Period</t>
+  </si>
+  <si>
+    <t>Course add/drop period</t>
+  </si>
+  <si>
+    <t>Midterm Exams Begin</t>
+  </si>
+  <si>
+    <t>Midterm examination period</t>
+  </si>
+  <si>
+    <t>Saint Elie Day</t>
+  </si>
+  <si>
+    <t>Public Holiday</t>
+  </si>
+  <si>
+    <t>Midterm Exams Begin TEST</t>
+  </si>
+  <si>
+    <t>Midterm examination period TEST</t>
+  </si>
+  <si>
+    <t>StartDay</t>
+  </si>
+  <si>
+    <t>StartMonth</t>
+  </si>
+  <si>
+    <t>StartYear</t>
+  </si>
+  <si>
+    <t>EndDay</t>
+  </si>
+  <si>
+    <t>EndMonth</t>
+  </si>
+  <si>
+    <t>EndYear</t>
   </si>
 </sst>
 </file>
@@ -188,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -197,9 +227,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -514,256 +554,536 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40EBC4DB-878C-491D-A5FD-57243F5A39BE}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="48.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="34.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.21875" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.77734375" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="C2" s="6">
+        <v>2</v>
+      </c>
+      <c r="D2" s="6">
+        <v>7</v>
+      </c>
+      <c r="E2" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="J2" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="4">
-        <v>46205</v>
-      </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3" t="s">
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="C3" s="6">
+        <v>6</v>
+      </c>
+      <c r="D3" s="6">
+        <v>7</v>
+      </c>
+      <c r="E3" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="J3" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="6">
+        <v>20</v>
+      </c>
+      <c r="D4" s="6">
+        <v>7</v>
+      </c>
+      <c r="E4" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F4" s="6">
+        <v>25</v>
+      </c>
+      <c r="G4" s="6">
+        <v>7</v>
+      </c>
+      <c r="H4" s="6">
+        <v>2026</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="6">
+        <v>5</v>
+      </c>
+      <c r="D5" s="6">
+        <v>8</v>
+      </c>
+      <c r="E5" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="6">
+        <v>15</v>
+      </c>
+      <c r="D6" s="6">
+        <v>8</v>
+      </c>
+      <c r="E6" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="4">
-        <v>46209</v>
-      </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3" t="s">
+      <c r="C7" s="7">
+        <v>13</v>
+      </c>
+      <c r="D7" s="7">
+        <v>1</v>
+      </c>
+      <c r="E7" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F7" s="7"/>
+      <c r="I7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="B8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="7">
+        <v>14</v>
+      </c>
+      <c r="D8" s="7">
+        <v>7</v>
+      </c>
+      <c r="E8" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F8" s="7"/>
+      <c r="I8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="7">
+        <v>15</v>
+      </c>
+      <c r="D9" s="7">
+        <v>7</v>
+      </c>
+      <c r="E9" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F9" s="7"/>
+      <c r="I9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="7">
+        <v>16</v>
+      </c>
+      <c r="D10" s="7">
+        <v>7</v>
+      </c>
+      <c r="E10" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F10" s="7"/>
+      <c r="I10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="7">
+        <v>20</v>
+      </c>
+      <c r="D11" s="7">
+        <v>7</v>
+      </c>
+      <c r="E11" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F11" s="7"/>
+      <c r="I11" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="7">
+        <v>31</v>
+      </c>
+      <c r="D12" s="7">
+        <v>7</v>
+      </c>
+      <c r="E12" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F12" s="7"/>
+      <c r="I12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="7">
+        <v>5</v>
+      </c>
+      <c r="D13" s="7">
+        <v>8</v>
+      </c>
+      <c r="E13" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F13" s="7"/>
+      <c r="I13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="7">
+        <v>15</v>
+      </c>
+      <c r="D14" s="7">
+        <v>8</v>
+      </c>
+      <c r="E14" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F14" s="7"/>
+      <c r="I14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="7">
+        <v>5</v>
+      </c>
+      <c r="D15" s="7">
+        <v>8</v>
+      </c>
+      <c r="E15" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F15" s="7"/>
+      <c r="I15" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="7">
+        <v>15</v>
+      </c>
+      <c r="D16" s="7">
+        <v>8</v>
+      </c>
+      <c r="E16" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F16" s="7"/>
+      <c r="I16" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="7">
+        <v>1</v>
+      </c>
+      <c r="D17" s="7">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="4">
-        <v>46211</v>
-      </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="E17" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F17" s="7"/>
+      <c r="I17" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="7">
+        <v>2</v>
+      </c>
+      <c r="D18" s="7">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="4">
-        <v>46212</v>
-      </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="4">
-        <v>46213</v>
-      </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="3" t="s">
+      <c r="E18" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F18" s="7"/>
+      <c r="I18" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="7">
         <v>20</v>
       </c>
-      <c r="C7" s="4">
-        <v>46216</v>
-      </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="4">
-        <v>46217</v>
-      </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="4">
-        <v>46218</v>
-      </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="4">
-        <v>46223</v>
-      </c>
-      <c r="D10" s="4">
-        <v>46228</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="4">
-        <v>46234</v>
-      </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="4">
-        <v>46239</v>
-      </c>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" s="4">
-        <v>46249</v>
-      </c>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>9</v>
+      <c r="D19" s="7">
+        <v>10</v>
+      </c>
+      <c r="E19" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F19" s="7"/>
+      <c r="I19" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="7">
+        <v>20</v>
+      </c>
+      <c r="D20" s="7">
+        <v>10</v>
+      </c>
+      <c r="E20" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F20" s="7">
+        <v>10</v>
+      </c>
+      <c r="G20" s="8">
+        <v>1</v>
+      </c>
+      <c r="H20" s="8">
+        <v>2027</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
entering 3 column for date start and end and updated VB accordingly
</commit_message>
<xml_diff>
--- a/App_Data/AcademicCalendar.xlsx
+++ b/App_Data/AcademicCalendar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elie.tawk\source\repos\AcademicCalendarProject\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{879C70B6-D5B2-4C5F-A3EB-80D4745EA5CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A74B5E34-174C-4502-B7CD-C0A9EA57E88A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{53C95AB7-0C09-47B5-9AE8-636C0202DA36}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="48">
   <si>
     <t>EventTitle</t>
   </si>
@@ -175,6 +175,12 @@
   </si>
   <si>
     <t>EndYear</t>
+  </si>
+  <si>
+    <t>ULS Entrance Exam for regular admission_TEST</t>
+  </si>
+  <si>
+    <t>Entrance exam for regular admission applicants_TEST</t>
   </si>
 </sst>
 </file>
@@ -554,7 +560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40EBC4DB-878C-491D-A5FD-57243F5A39BE}">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.88671875" style="2" bestFit="1" customWidth="1"/>
@@ -630,25 +636,31 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="C3" s="6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D3" s="6">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E3" s="5">
         <v>2026</v>
       </c>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
+      <c r="F3" s="6">
+        <v>31</v>
+      </c>
+      <c r="G3" s="6">
+        <v>4</v>
+      </c>
+      <c r="H3" s="6">
+        <v>2026</v>
+      </c>
       <c r="I3" s="3" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>6</v>
@@ -656,13 +668,13 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C4" s="6">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="D4" s="6">
         <v>7</v>
@@ -670,17 +682,11 @@
       <c r="E4" s="5">
         <v>2026</v>
       </c>
-      <c r="F4" s="6">
-        <v>25</v>
-      </c>
-      <c r="G4" s="6">
-        <v>7</v>
-      </c>
-      <c r="H4" s="6">
-        <v>2026</v>
-      </c>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
       <c r="I4" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>6</v>
@@ -688,25 +694,31 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C5" s="6">
+        <v>20</v>
+      </c>
+      <c r="D5" s="6">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F5" s="6">
+        <v>25</v>
+      </c>
+      <c r="G5" s="6">
+        <v>7</v>
+      </c>
+      <c r="H5" s="6">
+        <v>2026</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="D5" s="6">
-        <v>8</v>
-      </c>
-      <c r="E5" s="5">
-        <v>2026</v>
-      </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>6</v>
@@ -714,13 +726,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C6" s="6">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D6" s="6">
         <v>8</v>
@@ -732,7 +744,7 @@
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
       <c r="I6" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>6</v>
@@ -740,23 +752,25 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="7">
-        <v>13</v>
-      </c>
-      <c r="D7" s="7">
-        <v>1</v>
+        <v>25</v>
+      </c>
+      <c r="C7" s="6">
+        <v>15</v>
+      </c>
+      <c r="D7" s="6">
+        <v>8</v>
       </c>
       <c r="E7" s="5">
         <v>2026</v>
       </c>
-      <c r="F7" s="7"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
       <c r="I7" s="3" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>6</v>
@@ -764,23 +778,23 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="7">
         <v>13</v>
       </c>
-      <c r="C8" s="7">
-        <v>14</v>
-      </c>
       <c r="D8" s="7">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E8" s="5">
         <v>2026</v>
       </c>
       <c r="F8" s="7"/>
       <c r="I8" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J8" s="3" t="s">
         <v>6</v>
@@ -788,13 +802,13 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="7">
         <v>14</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="7">
-        <v>15</v>
       </c>
       <c r="D9" s="7">
         <v>7</v>
@@ -804,7 +818,7 @@
       </c>
       <c r="F9" s="7"/>
       <c r="I9" s="3" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="J9" s="3" t="s">
         <v>6</v>
@@ -812,13 +826,13 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C10" s="7">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D10" s="7">
         <v>7</v>
@@ -828,7 +842,7 @@
       </c>
       <c r="F10" s="7"/>
       <c r="I10" s="3" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>6</v>
@@ -836,13 +850,13 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="C11" s="7">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D11" s="7">
         <v>7</v>
@@ -852,7 +866,7 @@
       </c>
       <c r="F11" s="7"/>
       <c r="I11" s="3" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>6</v>
@@ -860,13 +874,13 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="7">
         <v>20</v>
-      </c>
-      <c r="C12" s="7">
-        <v>31</v>
       </c>
       <c r="D12" s="7">
         <v>7</v>
@@ -876,7 +890,7 @@
       </c>
       <c r="F12" s="7"/>
       <c r="I12" s="3" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>6</v>
@@ -884,23 +898,23 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C13" s="7">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="D13" s="7">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E13" s="5">
         <v>2026</v>
       </c>
       <c r="F13" s="7"/>
       <c r="I13" s="3" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>6</v>
@@ -908,13 +922,13 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C14" s="7">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D14" s="7">
         <v>8</v>
@@ -924,7 +938,7 @@
       </c>
       <c r="F14" s="7"/>
       <c r="I14" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>6</v>
@@ -932,13 +946,13 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C15" s="7">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D15" s="7">
         <v>8</v>
@@ -948,7 +962,7 @@
       </c>
       <c r="F15" s="7"/>
       <c r="I15" s="3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J15" s="3" t="s">
         <v>6</v>
@@ -956,13 +970,13 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C16" s="7">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D16" s="7">
         <v>8</v>
@@ -972,7 +986,7 @@
       </c>
       <c r="F16" s="7"/>
       <c r="I16" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>6</v>
@@ -980,23 +994,23 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C17" s="7">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D17" s="7">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E17" s="5">
         <v>2026</v>
       </c>
       <c r="F17" s="7"/>
       <c r="I17" s="3" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>6</v>
@@ -1004,13 +1018,13 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C18" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="7">
         <v>9</v>
@@ -1020,7 +1034,7 @@
       </c>
       <c r="F18" s="7"/>
       <c r="I18" s="3" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>6</v>
@@ -1028,23 +1042,23 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C19" s="7">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D19" s="7">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E19" s="5">
         <v>2026</v>
       </c>
       <c r="F19" s="7"/>
       <c r="I19" s="3" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>6</v>
@@ -1052,10 +1066,10 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C20" s="7">
         <v>20</v>
@@ -1066,19 +1080,43 @@
       <c r="E20" s="5">
         <v>2026</v>
       </c>
-      <c r="F20" s="7">
-        <v>10</v>
-      </c>
-      <c r="G20" s="8">
-        <v>1</v>
-      </c>
-      <c r="H20" s="8">
-        <v>2027</v>
-      </c>
+      <c r="F20" s="7"/>
       <c r="I20" s="3" t="s">
         <v>5</v>
       </c>
       <c r="J20" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="7">
+        <v>20</v>
+      </c>
+      <c r="D21" s="7">
+        <v>10</v>
+      </c>
+      <c r="E21" s="5">
+        <v>2026</v>
+      </c>
+      <c r="F21" s="7">
+        <v>10</v>
+      </c>
+      <c r="G21" s="8">
+        <v>1</v>
+      </c>
+      <c r="H21" s="8">
+        <v>2027</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J21" s="3" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>